<commit_message>
feat: implement batch persistence, dynamic pagination, and optimized R-language filtering to improve pipeline robustness and data extraction accuracy.
</commit_message>
<xml_diff>
--- a/coleta de dados gabriel.xlsx
+++ b/coleta de dados gabriel.xlsx
@@ -12931,17 +12931,17 @@
       </c>
       <c r="F2" s="23" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G2" s="22" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H2" s="22" t="inlineStr">
         <is>
-          <t>Websites de editoras (web scraping), Editoras diretamente (sob solicitação)</t>
+          <t>Web of Science, Scopus</t>
         </is>
       </c>
     </row>
@@ -13020,7 +13020,7 @@
       </c>
       <c r="G4" s="22" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H4" s="22" t="inlineStr">
@@ -13104,12 +13104,12 @@
       </c>
       <c r="G6" s="22" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H6" s="22" t="inlineStr">
         <is>
-          <t>Web of Science (WoS), Scopus</t>
+          <t>Web of Science, Scopus</t>
         </is>
       </c>
     </row>
@@ -13314,12 +13314,12 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Registros de doutorado de universidades holandesas, dados de publicação</t>
+          <t>Dutch university records</t>
         </is>
       </c>
     </row>
@@ -13403,7 +13403,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Literatura científica secundária (revisão sistemática de literatura), Literatura cinzenta</t>
+          <t>English-language sources, Russian literature, gray literature</t>
         </is>
       </c>
     </row>
@@ -13482,12 +13482,12 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Diretórios de periódicos de acesso aberto, dados de taxas de processamento de artigos (APCs)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -13566,12 +13566,12 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Dados de Butler et al. (2023), Web of Science (Peer Review gateway)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -13986,12 +13986,12 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>bioRxiv, medRxiv, arXiv, SSRN, 94 veículos de comunicação, Web of Science</t>
+          <t>bioRxiv, medRxiv, arXiv, SSRN, Web of Science</t>
         </is>
       </c>
     </row>
@@ -14868,12 +14868,12 @@
       </c>
       <c r="G48" s="22" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H48" s="22" t="inlineStr">
         <is>
-          <t>Artigo científico original e dados experimentais de Cruz-Castro &amp; Sanz-Menéndez (2023)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -14994,12 +14994,12 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Plataforma Sucupira, Plataforma Lattes (CNPq), Directory of Open Access Journals (DOAJ)</t>
+          <t>Plataforma Sucupira, Plataforma Lattes, Directory of Open Access Journals</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: update dataset entries with refined categorization and consistency flags
</commit_message>
<xml_diff>
--- a/coleta de dados gabriel.xlsx
+++ b/coleta de dados gabriel.xlsx
@@ -1169,12 +1169,12 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -1211,12 +1211,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1510,12 +1510,12 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Directory of Open Access Journals</t>
+          <t>Directory of Open Access Journals (DOAJ)</t>
         </is>
       </c>
     </row>
@@ -1920,12 +1920,12 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>large-scale text analysis</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2004,12 +2004,12 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>network-based approach</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>15 major Danish research funders</t>
+          <t>Danish research funders</t>
         </is>
       </c>
     </row>
@@ -2172,12 +2172,12 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>ORCID, Carnegie Classification</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>ORCID, Carnegie Classification of Institutions of Higher Education (CCIHE)</t>
+          <t>ORCID, Carnegie Classification of Institutions of Higher Education</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>ACPLC (Algorithmically constructed publication-level classification)</t>
+          <t>ACPLC, Construct</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -2434,12 +2434,12 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Canadian nanotechnology and advanced materials firms corporate websites</t>
+          <t>Corporate websites</t>
         </is>
       </c>
     </row>
@@ -2597,12 +2597,12 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
@@ -2639,12 +2639,12 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>2017 Journal Citation Reports of Clarivate Analytics</t>
+          <t>Clarivate Analytics</t>
         </is>
       </c>
     </row>
@@ -2728,12 +2728,12 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>open access journal articles</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>SwePub database</t>
+          <t>SwePub</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Stata (h_index), R (hindex)</t>
+          <t>Stata, R</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>visualização - gerar gráficos</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
@@ -3274,12 +3274,12 @@
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>PubMed Central (PMC)</t>
+          <t>PubMed Central</t>
         </is>
       </c>
     </row>
@@ -3306,12 +3306,12 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Citation Concept Analysis (CCA)</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>regressions</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>linear-time algorithms</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
@@ -3899,12 +3899,12 @@
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
@@ -3941,17 +3941,17 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>PhD theses</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -4020,12 +4020,12 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>agglomerative clustering method</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr">
@@ -4067,12 +4067,12 @@
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
@@ -4109,12 +4109,12 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H81" s="6" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
@@ -4277,12 +4277,12 @@
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>Web of Science, Scopus, Google Scholar</t>
+          <t>Google Scholar, Web of Science, Scopus</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>Scopus, MEDLINE</t>
+          <t>Scopus</t>
         </is>
       </c>
     </row>
@@ -4488,12 +4488,12 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>Scopus, Mendeley, Web of Science, MEDLINE</t>
+          <t>Scopus, Web of Science</t>
         </is>
       </c>
     </row>
@@ -4572,7 +4572,7 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
@@ -4807,7 +4807,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Deep learning</t>
+          <t>scite</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Elsevier</t>
+          <t>Elsevier’s Mirror Journal system</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -5190,12 +5190,12 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
@@ -5269,7 +5269,7 @@
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>Machine Learning, NLP</t>
+          <t>Machine Learning, Natural Language Processing</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -5442,12 +5442,12 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
@@ -5573,12 +5573,12 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Wikipedia, Web of Science, Crossref</t>
+          <t>Wikipedia, Crossref, Web of Science</t>
         </is>
       </c>
     </row>
@@ -5689,7 +5689,7 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>CERIF, RDC</t>
+          <t>Current Research Information Systems (CRIS), CERIF, RDC</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
@@ -5820,12 +5820,12 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
@@ -5862,12 +5862,12 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>coleta dos dados, análise dos dados, visualização - gerar gráficos</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>LIS journals</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -6035,7 +6035,7 @@
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H32" s="10" t="inlineStr">
@@ -6077,12 +6077,12 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>VABB-SHW, Cristin, Web of Science, Science-Metrix, ERIH PLUS</t>
+          <t>VABB-SHW, Cristin</t>
         </is>
       </c>
     </row>
@@ -6203,7 +6203,7 @@
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H36" s="10" t="inlineStr">
@@ -6413,12 +6413,12 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Patent data</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -6450,7 +6450,7 @@
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
@@ -6492,7 +6492,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -6534,17 +6534,17 @@
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>REF (Research Excellence Framework)</t>
+          <t>Research Excellence Framework (REF)</t>
         </is>
       </c>
     </row>
@@ -6576,12 +6576,12 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
@@ -6613,12 +6613,12 @@
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Poisson process model</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
@@ -6655,7 +6655,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>BIP4COVID19</t>
+          <t>keyword-based search interface</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados, visualização - gerar gráficos</t>
+          <t>análise dos dados, visualização - gerar gráficos</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
@@ -6744,12 +6744,12 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -6781,12 +6781,12 @@
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>social network analysis</t>
         </is>
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G50" s="10" t="inlineStr">
@@ -6823,22 +6823,22 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>rank-biased overlap, science overlay maps, clustering, heatmaps, network analytics</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados, visualização - gerar gráficos</t>
+          <t>análise dos dados, visualização - gerar gráficos</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Web of Science (WoS), Scopus, Chinese Science Citation Database (CSCD), Nature Index</t>
+          <t>Web of Science (WoS), Scopus, Chinese Science Citation Database (CSCD), Nature Index, Technology Alert List</t>
         </is>
       </c>
     </row>
@@ -7090,7 +7090,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>Chinese science citation database (CSCD)</t>
+          <t>Chinese Science Citation Database (CSCD)</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7159,7 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Vector Space Model, Latent Semantic Analysis, fastText, Random Indexing</t>
+          <t>fastText, Random Indexing (RI), Latent Semantic Analysis (LSA), Vector Space Model (VSM)</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
@@ -7589,7 +7589,7 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>análise dos dados, visualização - gerar gráficos</t>
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>EconGeo package for R</t>
+          <t>EconGeo (R package)</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
@@ -7841,7 +7841,7 @@
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H75" s="6" t="inlineStr">
@@ -8143,17 +8143,17 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ulrichsweb</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>Institutional documents</t>
+          <t>Documentação institucional</t>
         </is>
       </c>
     </row>
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>National universities (Italy)</t>
+          <t>Universidades italianas</t>
         </is>
       </c>
     </row>
@@ -8363,12 +8363,12 @@
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H10" s="14" t="inlineStr">
         <is>
-          <t>Academic databases (implied)</t>
+          <t>Scopus</t>
         </is>
       </c>
     </row>
@@ -8573,12 +8573,12 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Web</t>
         </is>
       </c>
     </row>
@@ -8620,7 +8620,7 @@
       </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t>Crossref, Web of Science, Scopus, Dimensions, Lens, PubMed</t>
+          <t>Crossref, Dutch Research Council, Web of Science, Scopus, Dimensions, Lens, PubMed</t>
         </is>
       </c>
     </row>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -8815,12 +8815,12 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Herfindahl-based index</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -8956,7 +8956,7 @@
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>Microsoft Academic Graph, Web of Science, Dimensions, ACM Digital Library</t>
+          <t>Microsoft Academic Graph, Web of Science (WoS), Dimensions, ACM Digital Library</t>
         </is>
       </c>
     </row>
@@ -8993,7 +8993,7 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados, visualização - gerar gráficos</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
@@ -9077,7 +9077,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
@@ -9203,7 +9203,7 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H30" s="14" t="inlineStr">
@@ -9235,17 +9235,17 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Microsoft Academic Graph, Crossref, OpenAIRE</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
@@ -9371,7 +9371,7 @@
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>visualização - gerar gráficos</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H34" s="14" t="inlineStr">
@@ -9413,7 +9413,7 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -9455,7 +9455,7 @@
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
@@ -9539,12 +9539,12 @@
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>American Economic Review</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -9581,7 +9581,7 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
@@ -9833,7 +9833,7 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
@@ -9875,7 +9875,7 @@
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H46" s="14" t="inlineStr">
@@ -9917,7 +9917,7 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
@@ -10001,7 +10001,7 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -10285,22 +10285,22 @@
       </c>
       <c r="E56" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sound level meter</t>
         </is>
       </c>
       <c r="F56" s="15" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H56" s="14" t="inlineStr">
         <is>
-          <t>GenBank</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="H58" s="14" t="inlineStr">
         <is>
-          <t>ICPSR</t>
+          <t>Interuniversity Consortium for Political and Social Research (ICPSR)</t>
         </is>
       </c>
     </row>
@@ -10998,17 +10998,17 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google Scholar</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -11055,7 +11055,7 @@
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>CNRS</t>
+          <t>Centre National de la Recherche Scientifique (CNRS)</t>
         </is>
       </c>
     </row>
@@ -11218,7 +11218,7 @@
       </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H16" s="18" t="inlineStr">
@@ -11376,12 +11376,12 @@
       </c>
       <c r="E20" s="18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="F20" s="19" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G20" s="18" t="inlineStr">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>MEDLINE</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>OECD</t>
+          <t>bibliometric data sources</t>
         </is>
       </c>
     </row>
@@ -11685,7 +11685,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Scopus, European Tertiary Education Register, SCImago Institutions Ranking</t>
+          <t>European Tertiary Education Register, SCImago Institutions Ranking, Scopus</t>
         </is>
       </c>
     </row>
@@ -11848,12 +11848,12 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Crossref, Scopus, ERIH PLUS</t>
+          <t>Crossref, ERIH PLUS, Scopus</t>
         </is>
       </c>
     </row>
@@ -11895,7 +11895,7 @@
       </c>
       <c r="H32" s="18" t="inlineStr">
         <is>
-          <t>Web of Science, Scopus, Dimensions, PubMed</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -11974,7 +11974,7 @@
       </c>
       <c r="G34" s="18" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados, visualização - gerar gráficos</t>
+          <t>visualização - gerar gráficos</t>
         </is>
       </c>
       <c r="H34" s="18" t="inlineStr">
@@ -12021,7 +12021,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Elsevier (Bibliographic data)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -12184,12 +12184,12 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Public health journals (h5 index data)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -12510,12 +12510,12 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Dictionary-based approach, embedding-enhanced query expansion</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -12557,12 +12557,12 @@
       </c>
       <c r="F48" s="19" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G48" s="18" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H48" s="18" t="inlineStr">
@@ -12594,7 +12594,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Coarsened exact matching</t>
+          <t>coarsened exact matching</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
@@ -12683,12 +12683,12 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
@@ -12720,17 +12720,17 @@
       </c>
       <c r="E52" s="18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>COUNTER R5, OpenURL link resolver</t>
         </is>
       </c>
       <c r="F52" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G52" s="18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H52" s="18" t="inlineStr">
@@ -15450,7 +15450,7 @@
       </c>
       <c r="F4" s="27" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G4" s="26" t="inlineStr">
@@ -15460,7 +15460,7 @@
       </c>
       <c r="H4" s="26" t="inlineStr">
         <is>
-          <t>Metadados de universidades (ranking e citações globais)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -15502,7 +15502,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Bases de dados bibliográficas (5 bases), Servidores de preprints (3 servidores)</t>
+          <t>bibliographic databases, preprint servers</t>
         </is>
       </c>
     </row>
@@ -15586,7 +15586,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Sistemas de Organização do Conhecimento (45 KOSs)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -15665,12 +15665,12 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Diretrizes de autores e declarações de acesso aberto de 300 periódicos</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -15707,12 +15707,12 @@
       </c>
       <c r="G10" s="26" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H10" s="26" t="inlineStr">
         <is>
-          <t>Retraction Watch, Amostra de 1 milhão de publicações</t>
+          <t>Retraction Watch</t>
         </is>
       </c>
     </row>
@@ -15749,7 +15749,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -16075,22 +16075,22 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>OpenAlex, Open Journal Systems</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>OpenAlex, Open Journal Systems (OJS), Crossref</t>
+          <t>OpenAlex</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Literatura científica secundária (Revisão teórica)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -16201,22 +16201,22 @@
       </c>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>PubPeer</t>
         </is>
       </c>
       <c r="F22" s="27" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G22" s="26" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H22" s="26" t="inlineStr">
         <is>
-          <t>Declarações de integridade de 117 universidades britânicas, PubPeer</t>
+          <t>PubPeer</t>
         </is>
       </c>
     </row>
@@ -16295,7 +16295,7 @@
       </c>
       <c r="G24" s="26" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H24" s="26" t="inlineStr">
@@ -16327,17 +16327,17 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>ORCID</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -16379,12 +16379,12 @@
       </c>
       <c r="G26" s="26" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H26" s="26" t="inlineStr">
         <is>
-          <t>Bases de dados bibliográficas (Scopus/Web of Science)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -16453,12 +16453,12 @@
       </c>
       <c r="E28" s="26" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Overton</t>
         </is>
       </c>
       <c r="F28" s="27" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G28" s="26" t="inlineStr">
@@ -16621,17 +16621,17 @@
       </c>
       <c r="E32" s="26" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Web of Science</t>
         </is>
       </c>
       <c r="F32" s="27" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G32" s="26" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H32" s="26" t="inlineStr">
@@ -16705,12 +16705,12 @@
       </c>
       <c r="E34" s="26" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>OpenAlex</t>
         </is>
       </c>
       <c r="F34" s="27" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G34" s="26" t="inlineStr">
@@ -16720,7 +16720,7 @@
       </c>
       <c r="H34" s="26" t="inlineStr">
         <is>
-          <t>OpenAlex, Scopus, Web of Science, African Journals Online (AJOL)</t>
+          <t>OpenAlex, Scopus, Web of Science, African Journals Online</t>
         </is>
       </c>
     </row>
@@ -16804,7 +16804,7 @@
       </c>
       <c r="H36" s="26" t="inlineStr">
         <is>
-          <t>N/A (Carta teórica e epistemológica)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -16883,12 +16883,12 @@
       </c>
       <c r="G38" s="26" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H38" s="26" t="inlineStr">
         <is>
-          <t>Websites da Clarivate, ISI e Thomson Reuters</t>
+          <t>Clarivate, Institute for Scientific Information, Thomson Reuters</t>
         </is>
       </c>
     </row>
@@ -17303,12 +17303,12 @@
       </c>
       <c r="G48" s="26" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H48" s="26" t="inlineStr">
         <is>
-          <t>Bases de dados bibliográficas (Scopus/Web of Science)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -17765,12 +17765,12 @@
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>14 agências de fomento públicas e privadas na Dinamarca</t>
+          <t>14 public and private research funders in Denmark</t>
         </is>
       </c>
     </row>
@@ -18136,12 +18136,12 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
         <is>
-          <t>Brapci</t>
+          <t>BRAPCI</t>
         </is>
       </c>
     </row>
@@ -18250,7 +18250,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -18288,7 +18288,7 @@
       </c>
       <c r="G8" s="30" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H8" s="30" t="inlineStr">
@@ -18402,12 +18402,12 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>UFSC</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -18473,12 +18473,12 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -18506,17 +18506,17 @@
       <c r="D14" s="30" t="inlineStr"/>
       <c r="E14" s="30" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Análise de Redes Sociais</t>
         </is>
       </c>
       <c r="F14" s="31" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G14" s="30" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H14" s="30" t="inlineStr">
@@ -18549,12 +18549,12 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -18587,12 +18587,12 @@
       </c>
       <c r="F16" s="31" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G16" s="30" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H16" s="30" t="inlineStr">
@@ -18663,12 +18663,12 @@
       </c>
       <c r="F18" s="31" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G18" s="30" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H18" s="30" t="inlineStr">
@@ -18701,12 +18701,12 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -18739,12 +18739,12 @@
       </c>
       <c r="F20" s="31" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G20" s="30" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H20" s="30" t="inlineStr">
@@ -18777,12 +18777,12 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -18924,7 +18924,7 @@
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Facebook, Twitter</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -18934,7 +18934,7 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -19015,7 +19015,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Web of Science, Scopus, Ranking de Leiden</t>
+          <t>Web of Science, Scopus</t>
         </is>
       </c>
     </row>
@@ -19086,7 +19086,7 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
@@ -19357,7 +19357,7 @@
       </c>
       <c r="H36" s="30" t="inlineStr">
         <is>
-          <t>Scientometrics</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Cadernos Pagu</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -19499,7 +19499,7 @@
       </c>
       <c r="F40" s="31" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G40" s="30" t="inlineStr">
@@ -19547,7 +19547,7 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Instituto Butantan</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -19841,12 +19841,12 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -20079,7 +20079,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>Censo da educação superior</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -20292,7 +20292,7 @@
       <c r="D61" s="6" t="inlineStr"/>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>LDA (Latent Dirichlet Allocation)</t>
+          <t>LDA</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
@@ -20307,7 +20307,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Periódicos internacionais</t>
         </is>
       </c>
     </row>
@@ -20459,7 +20459,7 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dados de orientações</t>
         </is>
       </c>
     </row>
@@ -20573,7 +20573,7 @@
       </c>
       <c r="H68" s="30" t="inlineStr">
         <is>
-          <t>Qualis CAPES</t>
+          <t>Periódicos brasileiros Qualis A1 e A2</t>
         </is>
       </c>
     </row>
@@ -20649,7 +20649,7 @@
       </c>
       <c r="H70" s="30" t="inlineStr">
         <is>
-          <t>ENANCIB</t>
+          <t>Enancib</t>
         </is>
       </c>
     </row>
@@ -20801,7 +20801,7 @@
       </c>
       <c r="H74" s="30" t="inlineStr">
         <is>
-          <t>ENANCIB</t>
+          <t>Enancib</t>
         </is>
       </c>
     </row>
@@ -20839,7 +20839,7 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>ENANCIB</t>
+          <t>Enancib</t>
         </is>
       </c>
     </row>
@@ -20877,7 +20877,7 @@
       </c>
       <c r="H76" s="30" t="inlineStr">
         <is>
-          <t>Biblioteca Comunitária (UFSCar)</t>
+          <t>Biblioteca Comunitária da Universidade Federal de São Carlos</t>
         </is>
       </c>
     </row>
@@ -20953,7 +20953,7 @@
       </c>
       <c r="H78" s="30" t="inlineStr">
         <is>
-          <t>Repositório Institucional da UFAM</t>
+          <t>RIU/UFAM</t>
         </is>
       </c>
     </row>
@@ -20991,7 +20991,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Anais de eventos</t>
+          <t>Anais de eventos nacionais</t>
         </is>
       </c>
     </row>
@@ -21029,7 +21029,7 @@
       </c>
       <c r="H80" s="30" t="inlineStr">
         <is>
-          <t>Teses e dissertações</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -21290,7 +21290,7 @@
       </c>
       <c r="G87" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados, visualização - gerar gráficos</t>
+          <t>análise dos dados, visualização - gerar gráficos</t>
         </is>
       </c>
       <c r="H87" s="6" t="inlineStr">
@@ -21366,12 +21366,12 @@
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>visualização - gerar gráficos</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>UFAM</t>
+          <t>Trabalhos de Conclusão de Curso (TCCs) da Universidade Federal do Amazonas (UFAM)</t>
         </is>
       </c>
     </row>
@@ -21901,7 +21901,7 @@
       </c>
       <c r="H8" s="34" t="inlineStr">
         <is>
-          <t>Fundação Oswaldo Cruz (Fiocruz)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -22064,7 +22064,7 @@
       </c>
       <c r="G12" s="34" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H12" s="34" t="inlineStr">
@@ -22180,12 +22180,12 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>cosseno de Salton</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -22232,7 +22232,7 @@
       </c>
       <c r="G16" s="34" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H16" s="34" t="inlineStr">
@@ -22279,7 +22279,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Portais de universidades federais</t>
+          <t>Portais de universidades</t>
         </is>
       </c>
     </row>
@@ -22363,7 +22363,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Enancib</t>
+          <t>ENANCIB</t>
         </is>
       </c>
     </row>
@@ -22437,12 +22437,12 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -22531,7 +22531,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Repositório Institucional</t>
+          <t>Repositório Institucional da UnB</t>
         </is>
       </c>
     </row>
@@ -22610,7 +22610,7 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -22652,7 +22652,7 @@
       </c>
       <c r="G26" s="34" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H26" s="34" t="inlineStr">
@@ -22736,7 +22736,7 @@
       </c>
       <c r="G28" s="34" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H28" s="34" t="inlineStr">
@@ -22778,12 +22778,12 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Plataforma Lattes, Web of Science, Journal Citation Reports, Qualis Periódicos</t>
+          <t>Plataforma Lattes</t>
         </is>
       </c>
     </row>
@@ -22820,7 +22820,7 @@
       </c>
       <c r="G30" s="34" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H30" s="34" t="inlineStr">
@@ -22862,7 +22862,7 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
@@ -23035,7 +23035,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>SCOPUS</t>
+          <t>Scopus</t>
         </is>
       </c>
     </row>
@@ -23245,7 +23245,7 @@
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
-          <t>Periódicos</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -23366,12 +23366,12 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Plataforma Lattes, CNPq</t>
+          <t>Plataforma Lattes</t>
         </is>
       </c>
     </row>
@@ -23408,7 +23408,7 @@
       </c>
       <c r="G44" s="34" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H44" s="34" t="inlineStr">
@@ -23492,7 +23492,7 @@
       </c>
       <c r="G46" s="34" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H46" s="34" t="inlineStr">
@@ -23534,7 +23534,7 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
@@ -23576,7 +23576,7 @@
       </c>
       <c r="G48" s="34" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H48" s="34" t="inlineStr">
@@ -23618,7 +23618,7 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -23697,7 +23697,7 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -23749,7 +23749,7 @@
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
-          <t>bases de dados</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -23870,7 +23870,7 @@
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
@@ -23954,7 +23954,7 @@
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
@@ -23996,7 +23996,7 @@
       </c>
       <c r="G58" s="34" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H58" s="34" t="inlineStr">
@@ -24127,7 +24127,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Plataforma Sucupira, Qualis-CAPES</t>
+          <t>Plataforma Sucupira</t>
         </is>
       </c>
     </row>
@@ -24169,7 +24169,7 @@
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
-          <t>CAPES, Latindex</t>
+          <t>Latindex, Qualis Periódicos</t>
         </is>
       </c>
     </row>
@@ -24248,7 +24248,7 @@
       </c>
       <c r="G64" s="34" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H64" s="34" t="inlineStr">
@@ -24290,7 +24290,7 @@
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr">
@@ -24374,7 +24374,7 @@
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr">
@@ -24500,12 +24500,12 @@
       </c>
       <c r="G70" s="34" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
-          <t>BRAPCI</t>
+          <t>Base de dados em Ciência da Informação</t>
         </is>
       </c>
     </row>
@@ -24542,12 +24542,12 @@
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>BRAPCI</t>
+          <t>Brapci</t>
         </is>
       </c>
     </row>
@@ -24663,12 +24663,12 @@
       </c>
       <c r="F74" s="35" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G74" s="34" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H74" s="34" t="inlineStr">
@@ -24705,12 +24705,12 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H75" s="6" t="inlineStr">
@@ -24757,7 +24757,7 @@
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
-          <t>IBICT</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -24789,12 +24789,12 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H77" s="6" t="inlineStr">
@@ -24925,7 +24925,7 @@
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Portais oficiais de periódicos, mídias sociais</t>
         </is>
       </c>
     </row>
@@ -24957,12 +24957,12 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H81" s="6" t="inlineStr">
@@ -24999,12 +24999,12 @@
       </c>
       <c r="F82" s="35" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G82" s="34" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H82" s="34" t="inlineStr">
@@ -25256,7 +25256,7 @@
       </c>
       <c r="G88" s="34" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H88" s="34" t="inlineStr">
@@ -25544,7 +25544,7 @@
       </c>
       <c r="H4" s="38" t="inlineStr">
         <is>
-          <t>Catálogo de Teses e Dissertações (CAPES)</t>
+          <t>Teses e dissertações brasileiras</t>
         </is>
       </c>
     </row>
@@ -25670,7 +25670,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>RICI (site)</t>
+          <t>Site da RICI</t>
         </is>
       </c>
     </row>
@@ -25749,12 +25749,12 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Planos de ensino de cursos de graduação em Biblioteconomia no Brasil</t>
+          <t>Planos de ensino de cursos de graduação em Biblioteconomia</t>
         </is>
       </c>
     </row>
@@ -25796,7 +25796,7 @@
       </c>
       <c r="H10" s="38" t="inlineStr">
         <is>
-          <t>Bases de dados científicas</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -25838,7 +25838,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Bases de dados científicas</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -25907,22 +25907,22 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>GitHub, FigShare</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Altmetric TOP 100, GitHub, FigShare</t>
+          <t>Altmetric TOP 100</t>
         </is>
       </c>
     </row>
@@ -26001,7 +26001,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -26132,7 +26132,7 @@
       </c>
       <c r="H18" s="38" t="inlineStr">
         <is>
-          <t>Repositório Lume, ResearchGate</t>
+          <t>ResearchGate, Repositório Lume</t>
         </is>
       </c>
     </row>
@@ -26416,12 +26416,12 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>coleta dos dados, visualização - gerar gráficos</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -26636,7 +26636,7 @@
       </c>
       <c r="H30" s="38" t="inlineStr">
         <is>
-          <t>Bases de dados de C&amp;T</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -26668,12 +26668,12 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
@@ -26715,12 +26715,12 @@
       </c>
       <c r="G32" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H32" s="38" t="inlineStr">
         <is>
-          <t>Repositórios Institucionais, Web social</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -26757,12 +26757,12 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Portal OASISBR</t>
+          <t>OASISBR</t>
         </is>
       </c>
     </row>
@@ -26799,7 +26799,7 @@
       </c>
       <c r="G34" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H34" s="38" t="inlineStr">
@@ -26831,17 +26831,17 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lei de Zipf</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -26883,12 +26883,12 @@
       </c>
       <c r="G36" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H36" s="38" t="inlineStr">
         <is>
-          <t>Poder Executivo Municipal</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -26925,7 +26925,7 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
@@ -27177,7 +27177,7 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
@@ -27261,7 +27261,7 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
@@ -27303,12 +27303,12 @@
       </c>
       <c r="G46" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H46" s="38" t="inlineStr">
         <is>
-          <t>Lattes</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -27387,7 +27387,7 @@
       </c>
       <c r="G48" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H48" s="38" t="inlineStr">
@@ -27429,7 +27429,7 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -27602,7 +27602,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>CoARA</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -27629,12 +27629,12 @@
       </c>
       <c r="E54" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>leis bibliométricas de Zipf</t>
         </is>
       </c>
       <c r="F54" s="39" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G54" s="38" t="inlineStr">
@@ -27676,12 +27676,12 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
@@ -27770,7 +27770,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>Dedalus, Web of Science</t>
+          <t>Dedalus (USP), Web of Science</t>
         </is>
       </c>
     </row>
@@ -27802,17 +27802,17 @@
       </c>
       <c r="F58" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G58" s="38" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H58" s="38" t="inlineStr">
         <is>
-          <t>Twitter (X), BRAPCI, Qualis Capes</t>
+          <t>BRAPCI, Twitter (X)</t>
         </is>
       </c>
     </row>
@@ -27844,17 +27844,17 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Plataforma Lattes</t>
         </is>
       </c>
     </row>
@@ -27896,7 +27896,7 @@
       </c>
       <c r="H60" s="38" t="inlineStr">
         <is>
-          <t>SisGen</t>
+          <t>Sisgen</t>
         </is>
       </c>
     </row>
@@ -27928,7 +27928,7 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -27965,12 +27965,12 @@
       </c>
       <c r="E62" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Social Network Analysis</t>
         </is>
       </c>
       <c r="F62" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G62" s="38" t="inlineStr">
@@ -28133,12 +28133,12 @@
       </c>
       <c r="E66" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>OpenAlex</t>
         </is>
       </c>
       <c r="F66" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G66" s="38" t="inlineStr">
@@ -28148,7 +28148,7 @@
       </c>
       <c r="H66" s="38" t="inlineStr">
         <is>
-          <t>OpenAlex, Qualis</t>
+          <t>OpenAlex</t>
         </is>
       </c>
     </row>
@@ -28185,7 +28185,7 @@
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr">
@@ -28311,12 +28311,12 @@
       </c>
       <c r="G70" s="38" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H70" s="38" t="inlineStr">
         <is>
-          <t>Websites institucionais (PUC)</t>
+          <t>Websites das bibliotecas</t>
         </is>
       </c>
     </row>
@@ -28353,7 +28353,7 @@
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr">
@@ -28437,12 +28437,12 @@
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Altmetric</t>
         </is>
       </c>
     </row>
@@ -28474,7 +28474,7 @@
       </c>
       <c r="F74" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G74" s="38" t="inlineStr">
@@ -28516,7 +28516,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
@@ -28600,7 +28600,7 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
@@ -28684,7 +28684,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr">
@@ -28694,7 +28694,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Planos de ensino</t>
         </is>
       </c>
     </row>
@@ -28862,7 +28862,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>Brapci, Plataforma Lattes</t>
+          <t>Brapci, LinkedIn</t>
         </is>
       </c>
     </row>
@@ -28894,12 +28894,12 @@
       </c>
       <c r="F84" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G84" s="38" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H84" s="38" t="inlineStr">
@@ -28988,7 +28988,7 @@
       </c>
       <c r="H86" s="38" t="inlineStr">
         <is>
-          <t>Plataforma Lattes, Painel de Dados CAPES</t>
+          <t>Plataforma Lattes, Painel de Dados da CAPES</t>
         </is>
       </c>
     </row>
@@ -29030,7 +29030,7 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>Periódicos Científicos</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -29062,12 +29062,12 @@
       </c>
       <c r="F88" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G88" s="38" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H88" s="38" t="inlineStr">
@@ -29104,12 +29104,12 @@
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H89" s="6" t="inlineStr">
@@ -29183,17 +29183,17 @@
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>SERVQual, Método Kano</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr">
@@ -29314,7 +29314,7 @@
       </c>
       <c r="F94" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G94" s="38" t="inlineStr">
@@ -29398,12 +29398,12 @@
       </c>
       <c r="F96" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G96" s="38" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>coleta dos dados</t>
         </is>
       </c>
       <c r="H96" s="38" t="inlineStr">
@@ -29608,7 +29608,7 @@
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G101" s="6" t="inlineStr">
@@ -29645,17 +29645,17 @@
       </c>
       <c r="E102" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Negative binomial regression</t>
         </is>
       </c>
       <c r="F102" s="39" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G102" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H102" s="38" t="inlineStr">
@@ -29949,7 +29949,7 @@
       </c>
       <c r="G109" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados, visualização - gerar gráficos</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H109" s="6" t="inlineStr">
@@ -30075,7 +30075,7 @@
       </c>
       <c r="G112" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H112" s="38" t="inlineStr">
@@ -30117,7 +30117,7 @@
       </c>
       <c r="G113" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H113" s="6" t="inlineStr">
@@ -30159,12 +30159,12 @@
       </c>
       <c r="G114" s="38" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H114" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BENANCIB</t>
         </is>
       </c>
     </row>
@@ -30243,7 +30243,7 @@
       </c>
       <c r="G116" s="38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>coleta dos dados, análise dos dados</t>
         </is>
       </c>
       <c r="H116" s="38" t="inlineStr">
@@ -30285,7 +30285,7 @@
       </c>
       <c r="G117" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H117" s="6" t="inlineStr">
@@ -30327,12 +30327,12 @@
       </c>
       <c r="G118" s="38" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H118" s="38" t="inlineStr">
         <is>
-          <t>Web of Science, Brapci</t>
+          <t>WoS, BRAPCI</t>
         </is>
       </c>
     </row>
@@ -30490,12 +30490,12 @@
       </c>
       <c r="F122" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G122" s="38" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H122" s="38" t="inlineStr">
@@ -30611,12 +30611,12 @@
       </c>
       <c r="E125" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Negative binomial regression</t>
         </is>
       </c>
       <c r="F125" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G125" s="6" t="inlineStr">
@@ -30626,7 +30626,7 @@
       </c>
       <c r="H125" s="6" t="inlineStr">
         <is>
-          <t>Scopus, Web of Science</t>
+          <t>Scopus, WoS</t>
         </is>
       </c>
     </row>
@@ -30705,12 +30705,12 @@
       </c>
       <c r="G127" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H127" s="6" t="inlineStr">
         <is>
-          <t>Centro de Memória da Amazônia da Universidade Federal do Pará, Arquivo Público do Pará</t>
+          <t>Centro de Memória da Amazônia da UFPA, Arquivo Público do Pará</t>
         </is>
       </c>
     </row>
@@ -30784,12 +30784,12 @@
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G129" s="6" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H129" s="6" t="inlineStr">
@@ -30826,12 +30826,12 @@
       </c>
       <c r="F130" s="39" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G130" s="38" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H130" s="38" t="inlineStr">
@@ -30868,17 +30868,17 @@
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G131" s="6" t="inlineStr">
         <is>
-          <t>coleta dos dados, análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
-          <t>CNPq</t>
+          <t>Plataforma Lattes</t>
         </is>
       </c>
     </row>
@@ -31167,7 +31167,7 @@
       </c>
       <c r="G138" s="38" t="inlineStr">
         <is>
-          <t>visualização - gerar gráficos</t>
+          <t>análise dos dados, visualização - gerar gráficos</t>
         </is>
       </c>
       <c r="H138" s="38" t="inlineStr">

</xml_diff>

<commit_message>
feat: add correspondence analysis script, generated biplot, and refine datasets
</commit_message>
<xml_diff>
--- a/coleta de dados gabriel.xlsx
+++ b/coleta de dados gabriel.xlsx
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'QSS 2020'!$A$1:$H$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QSS 2021'!$A$1:$H$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'QSS 2022'!$A$1:$H$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'QSS 2022'!$A$1:$H$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'QSS 2023'!$A$1:$H$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'QSS 2024'!$A$1:$H$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'QSS 2025'!$A$1:$H$62</definedName>
@@ -7939,7 +7939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -10265,37 +10265,37 @@
     <row r="56" ht="24" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1162/qss_a_00181</t>
+          <t>https://doi.org/10.1162/qss_a_00186</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Traffic Noise, Hazardous noise level, Kurnool city, NIHL, Ambient Noise level, Health education, Sound level meter.</t>
+          <t>See further upon the giants: Quantifying intellectual lineage in science</t>
         </is>
       </c>
       <c r="C56" s="14" t="inlineStr">
         <is>
-          <t>C. Sunil Kumar, Salman Ahmed, M. Mahendra Kumar, H N Champa, M.S. Prakash Rao, Gulnaz Hameed</t>
+          <t>Woo Seong Jo, Lu Liu, Dashun Wang</t>
         </is>
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>Sound level meter, Noise (video), Noise level, Hazardous waste, Ambient noise level, Metre, Noise exposure, Environmental science, Background noise, Traffic noise, Acoustics, Sound (geography), Hearing loss, Audiology, Engineering, Medicine, Computer science, Noise reduction, Physics, Waste management</t>
+          <t>Citation, Shoulders, Index (typography), Dimension (graph theory), Computer science, Library science, Mathematics, Medicine</t>
         </is>
       </c>
       <c r="E56" s="14" t="inlineStr">
         <is>
-          <t>Sound level meter</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F56" s="15" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
-          <t>coleta dos dados</t>
+          <t>análise dos dados</t>
         </is>
       </c>
       <c r="H56" s="14" t="inlineStr">
@@ -10307,22 +10307,22 @@
     <row r="57" ht="24" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1162/qss_a_00186</t>
+          <t>https://doi.org/10.1162/qss_a_00209</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>See further upon the giants: Quantifying intellectual lineage in science</t>
+          <t>Subdivisions and crossroads: Identifying hidden community structures in a data archive’s citation network</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Woo Seong Jo, Lu Liu, Dashun Wang</t>
+          <t>Sara Lafia, Lizhou Fan, Andrea K. Thomer, Libby Hemphill</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Citation, Shoulders, Index (typography), Dimension (graph theory), Computer science, Library science, Mathematics, Medicine</t>
+          <t>Citation, Reuse, Data science, Social network analysis, Computer science, Discipline, Social network (sociolinguistics), World Wide Web, Sociology, Social media, Social science, Engineering</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
@@ -10342,29 +10342,25 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Interuniversity Consortium for Political and Social Research (ICPSR)</t>
         </is>
       </c>
     </row>
     <row r="58" ht="24" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1162/qss_a_00209</t>
+          <t>https://doi.org/10.1162/qss_e_00196</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Subdivisions and crossroads: Identifying hidden community structures in a data archive’s citation network</t>
-        </is>
-      </c>
-      <c r="C58" s="14" t="inlineStr">
-        <is>
-          <t>Sara Lafia, Lizhou Fan, Andrea K. Thomer, Libby Hemphill</t>
-        </is>
-      </c>
+          <t>Erratum</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr"/>
       <c r="D58" s="14" t="inlineStr">
         <is>
-          <t>Citation, Reuse, Data science, Social network analysis, Computer science, Discipline, Social network (sociolinguistics), World Wide Web, Sociology, Social media, Social science, Engineering</t>
+          <t>License, Citation, Icon, Download, Computer science, Information retrieval, World Wide Web, Library science</t>
         </is>
       </c>
       <c r="E58" s="14" t="inlineStr">
@@ -10374,35 +10370,39 @@
       </c>
       <c r="F58" s="15" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G58" s="14" t="inlineStr">
         <is>
-          <t>análise dos dados</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H58" s="14" t="inlineStr">
         <is>
-          <t>Interuniversity Consortium for Political and Social Research (ICPSR)</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="59" ht="24" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1162/qss_e_00196</t>
+          <t>https://doi.org/10.1162/qss_c_00197</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Erratum</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr"/>
+          <t>Values matter in science, so do facts: Response to Gingras</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Kyle Siler</t>
+        </is>
+      </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>License, Citation, Icon, Download, Computer science, Information retrieval, World Wide Web, Library science</t>
+          <t>License, Citation, Icon, Library science, Attribution, History, Computer science, Political science, Law, Psychology</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
@@ -10426,50 +10426,8 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="24" customHeight="1">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1162/qss_c_00197</t>
-        </is>
-      </c>
-      <c r="B60" s="14" t="inlineStr">
-        <is>
-          <t>Values matter in science, so do facts: Response to Gingras</t>
-        </is>
-      </c>
-      <c r="C60" s="14" t="inlineStr">
-        <is>
-          <t>Kyle Siler</t>
-        </is>
-      </c>
-      <c r="D60" s="14" t="inlineStr">
-        <is>
-          <t>License, Citation, Icon, Library science, Attribution, History, Computer science, Political science, Law, Psychology</t>
-        </is>
-      </c>
-      <c r="E60" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F60" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G60" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H60" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H60"/>
+  <autoFilter ref="A1:H59"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -10529,7 +10487,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>